<commit_message>
update xlsx to fix corruption issue
In commit 2363398, a single cell with a font definition longer
than 31 characters (the max Excel accepts) was accidentally
introduced. This went unnoticed, because LibreOffice does not
have such a limitation.

The issue was resolved by just painting the style of the adjacent
cell over the affected one, G627, /Luminosity.
</commit_message>
<xml_diff>
--- a/CCGX-Modbus-TCP-register-list.xlsx
+++ b/CCGX-Modbus-TCP-register-list.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Field list" sheetId="1" state="visible" r:id="rId3"/>
@@ -5677,7 +5677,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -5735,13 +5735,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Liberation Mono;Courier New;DejaVu Sans Mono;Monaco"/>
-      <family val="3"/>
       <charset val="1"/>
     </font>
     <font>
@@ -5860,7 +5853,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5978,10 +5971,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5993,7 +5982,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -24396,7 +24385,7 @@
       <c r="F627" s="3" t="s">
         <v>1215</v>
       </c>
-      <c r="G627" s="29" t="s">
+      <c r="G627" s="1" t="s">
         <v>1216</v>
       </c>
       <c r="H627" s="1" t="s">
@@ -25764,7 +25753,7 @@
       <c r="E678" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F678" s="30" t="s">
+      <c r="F678" s="29" t="s">
         <v>750</v>
       </c>
       <c r="G678" s="1" t="s">
@@ -25822,7 +25811,7 @@
       <c r="E680" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="F680" s="31" t="s">
+      <c r="F680" s="30" t="s">
         <v>1307</v>
       </c>
       <c r="G680" s="1" t="s">
@@ -25848,7 +25837,7 @@
       <c r="E681" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="F681" s="31" t="s">
+      <c r="F681" s="30" t="s">
         <v>1307</v>
       </c>
       <c r="G681" s="1" t="s">
@@ -26339,13 +26328,13 @@
       <c r="C700" s="1" t="n">
         <v>3924</v>
       </c>
-      <c r="D700" s="32" t="s">
+      <c r="D700" s="31" t="s">
         <v>136</v>
       </c>
       <c r="E700" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F700" s="31" t="s">
+      <c r="F700" s="30" t="s">
         <v>140</v>
       </c>
       <c r="G700" s="1" t="s">
@@ -26368,13 +26357,13 @@
       <c r="C701" s="1" t="n">
         <v>3926</v>
       </c>
-      <c r="D701" s="32" t="s">
+      <c r="D701" s="31" t="s">
         <v>136</v>
       </c>
       <c r="E701" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F701" s="31" t="s">
+      <c r="F701" s="30" t="s">
         <v>140</v>
       </c>
       <c r="G701" s="1" t="s">
@@ -26397,13 +26386,13 @@
       <c r="C702" s="1" t="n">
         <v>3928</v>
       </c>
-      <c r="D702" s="32" t="s">
+      <c r="D702" s="31" t="s">
         <v>136</v>
       </c>
       <c r="E702" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F702" s="31" t="s">
+      <c r="F702" s="30" t="s">
         <v>140</v>
       </c>
       <c r="G702" s="1" t="s">
@@ -26564,7 +26553,7 @@
       <c r="C709" s="22" t="n">
         <v>4000</v>
       </c>
-      <c r="D709" s="32" t="s">
+      <c r="D709" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E709" s="22" t="n">
@@ -26593,7 +26582,7 @@
       <c r="C710" s="22" t="n">
         <v>4001</v>
       </c>
-      <c r="D710" s="32" t="s">
+      <c r="D710" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E710" s="22" t="n">
@@ -26622,7 +26611,7 @@
       <c r="C711" s="22" t="n">
         <v>4002</v>
       </c>
-      <c r="D711" s="32" t="s">
+      <c r="D711" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E711" s="22" t="n">
@@ -26651,7 +26640,7 @@
       <c r="C712" s="22" t="n">
         <v>4003</v>
       </c>
-      <c r="D712" s="32" t="s">
+      <c r="D712" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E712" s="22" t="n">
@@ -26680,7 +26669,7 @@
       <c r="C713" s="22" t="n">
         <v>4004</v>
       </c>
-      <c r="D713" s="32" t="s">
+      <c r="D713" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E713" s="22" t="n">
@@ -26709,7 +26698,7 @@
       <c r="C714" s="22" t="n">
         <v>4006</v>
       </c>
-      <c r="D714" s="32" t="s">
+      <c r="D714" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E714" s="22" t="n">
@@ -26738,7 +26727,7 @@
       <c r="C715" s="22" t="n">
         <v>4007</v>
       </c>
-      <c r="D715" s="32" t="s">
+      <c r="D715" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E715" s="22" t="n">
@@ -26767,7 +26756,7 @@
       <c r="C716" s="22" t="n">
         <v>4008</v>
       </c>
-      <c r="D716" s="32" t="s">
+      <c r="D716" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E716" s="22" t="n">
@@ -26796,7 +26785,7 @@
       <c r="C717" s="22" t="n">
         <v>4009</v>
       </c>
-      <c r="D717" s="32" t="s">
+      <c r="D717" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E717" s="22" t="n">
@@ -26825,7 +26814,7 @@
       <c r="C718" s="22" t="n">
         <v>4010</v>
       </c>
-      <c r="D718" s="32" t="s">
+      <c r="D718" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E718" s="22" t="n">
@@ -26854,7 +26843,7 @@
       <c r="C719" s="22" t="n">
         <v>4011</v>
       </c>
-      <c r="D719" s="32" t="s">
+      <c r="D719" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E719" s="22" t="n">
@@ -26883,7 +26872,7 @@
       <c r="C720" s="22" t="n">
         <v>4100</v>
       </c>
-      <c r="D720" s="32" t="s">
+      <c r="D720" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E720" s="22" t="n">
@@ -26912,7 +26901,7 @@
       <c r="C721" s="22" t="n">
         <v>4101</v>
       </c>
-      <c r="D721" s="32" t="s">
+      <c r="D721" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E721" s="22" t="n">
@@ -26941,7 +26930,7 @@
       <c r="C722" s="22" t="n">
         <v>4102</v>
       </c>
-      <c r="D722" s="32" t="s">
+      <c r="D722" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E722" s="22" t="n">
@@ -26970,7 +26959,7 @@
       <c r="C723" s="22" t="n">
         <v>4103</v>
       </c>
-      <c r="D723" s="32" t="s">
+      <c r="D723" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E723" s="22" t="n">
@@ -26999,7 +26988,7 @@
       <c r="C724" s="22" t="n">
         <v>4104</v>
       </c>
-      <c r="D724" s="32" t="s">
+      <c r="D724" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E724" s="22" t="n">
@@ -27028,7 +27017,7 @@
       <c r="C725" s="22" t="n">
         <v>4106</v>
       </c>
-      <c r="D725" s="32" t="s">
+      <c r="D725" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E725" s="22" t="n">
@@ -27057,7 +27046,7 @@
       <c r="C726" s="22" t="n">
         <v>4107</v>
       </c>
-      <c r="D726" s="32" t="s">
+      <c r="D726" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E726" s="22" t="n">
@@ -27086,7 +27075,7 @@
       <c r="C727" s="22" t="n">
         <v>4108</v>
       </c>
-      <c r="D727" s="32" t="s">
+      <c r="D727" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E727" s="22" t="n">
@@ -27115,7 +27104,7 @@
       <c r="C728" s="22" t="n">
         <v>4109</v>
       </c>
-      <c r="D728" s="32" t="s">
+      <c r="D728" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E728" s="22" t="n">
@@ -27144,7 +27133,7 @@
       <c r="C729" s="22" t="n">
         <v>4110</v>
       </c>
-      <c r="D729" s="32" t="s">
+      <c r="D729" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E729" s="22" t="n">
@@ -27173,7 +27162,7 @@
       <c r="C730" s="22" t="n">
         <v>4111</v>
       </c>
-      <c r="D730" s="32" t="s">
+      <c r="D730" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E730" s="22" t="n">
@@ -27202,7 +27191,7 @@
       <c r="C731" s="22" t="n">
         <v>4112</v>
       </c>
-      <c r="D731" s="32" t="s">
+      <c r="D731" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E731" s="22" t="n">
@@ -27231,7 +27220,7 @@
       <c r="C732" s="22" t="n">
         <v>4113</v>
       </c>
-      <c r="D732" s="32" t="s">
+      <c r="D732" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E732" s="22" t="n">
@@ -27260,7 +27249,7 @@
       <c r="C733" s="22" t="n">
         <v>4114</v>
       </c>
-      <c r="D733" s="32" t="s">
+      <c r="D733" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E733" s="22" t="n">
@@ -27289,7 +27278,7 @@
       <c r="C734" s="22" t="n">
         <v>4115</v>
       </c>
-      <c r="D734" s="32" t="s">
+      <c r="D734" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E734" s="22" t="n">
@@ -27318,7 +27307,7 @@
       <c r="C735" s="22" t="n">
         <v>4116</v>
       </c>
-      <c r="D735" s="32" t="s">
+      <c r="D735" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E735" s="22" t="n">
@@ -27347,7 +27336,7 @@
       <c r="C736" s="22" t="n">
         <v>4117</v>
       </c>
-      <c r="D736" s="32" t="s">
+      <c r="D736" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E736" s="22" t="n">
@@ -27376,7 +27365,7 @@
       <c r="C737" s="22" t="n">
         <v>4118</v>
       </c>
-      <c r="D737" s="32" t="s">
+      <c r="D737" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E737" s="22" t="n">
@@ -27405,7 +27394,7 @@
       <c r="C738" s="22" t="n">
         <v>4119</v>
       </c>
-      <c r="D738" s="32" t="s">
+      <c r="D738" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E738" s="22" t="n">
@@ -27434,7 +27423,7 @@
       <c r="C739" s="22" t="n">
         <v>4120</v>
       </c>
-      <c r="D739" s="32" t="s">
+      <c r="D739" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E739" s="22" t="n">
@@ -27463,7 +27452,7 @@
       <c r="C740" s="22" t="s">
         <v>1338</v>
       </c>
-      <c r="D740" s="32"/>
+      <c r="D740" s="31"/>
       <c r="E740" s="22"/>
       <c r="G740" s="22" t="s">
         <v>117</v>
@@ -27479,7 +27468,7 @@
       <c r="C741" s="22" t="n">
         <v>4220</v>
       </c>
-      <c r="D741" s="32" t="s">
+      <c r="D741" s="31" t="s">
         <v>440</v>
       </c>
       <c r="E741" s="22"/>
@@ -27500,7 +27489,7 @@
       <c r="C742" s="22" t="n">
         <v>4200</v>
       </c>
-      <c r="D742" s="32" t="s">
+      <c r="D742" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E742" s="22" t="n">
@@ -27529,7 +27518,7 @@
       <c r="C743" s="22" t="n">
         <v>4201</v>
       </c>
-      <c r="D743" s="32" t="s">
+      <c r="D743" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E743" s="22" t="n">
@@ -27558,7 +27547,7 @@
       <c r="C744" s="22" t="n">
         <v>4202</v>
       </c>
-      <c r="D744" s="32" t="s">
+      <c r="D744" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E744" s="22" t="n">
@@ -27587,7 +27576,7 @@
       <c r="C745" s="22" t="n">
         <v>4203</v>
       </c>
-      <c r="D745" s="32" t="s">
+      <c r="D745" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E745" s="22" t="n">
@@ -27616,7 +27605,7 @@
       <c r="C746" s="22" t="n">
         <v>4204</v>
       </c>
-      <c r="D746" s="32" t="s">
+      <c r="D746" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E746" s="22" t="n">
@@ -27645,7 +27634,7 @@
       <c r="C747" s="22" t="n">
         <v>4206</v>
       </c>
-      <c r="D747" s="32" t="s">
+      <c r="D747" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E747" s="22" t="n">
@@ -27674,7 +27663,7 @@
       <c r="C748" s="22" t="n">
         <v>4207</v>
       </c>
-      <c r="D748" s="32" t="s">
+      <c r="D748" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E748" s="22" t="n">
@@ -27703,7 +27692,7 @@
       <c r="C749" s="22" t="n">
         <v>4208</v>
       </c>
-      <c r="D749" s="32" t="s">
+      <c r="D749" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E749" s="22" t="n">
@@ -27732,7 +27721,7 @@
       <c r="C750" s="22" t="n">
         <v>4209</v>
       </c>
-      <c r="D750" s="32" t="s">
+      <c r="D750" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E750" s="22" t="n">
@@ -27761,7 +27750,7 @@
       <c r="C751" s="22" t="n">
         <v>4210</v>
       </c>
-      <c r="D751" s="32" t="s">
+      <c r="D751" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E751" s="22" t="n">
@@ -27790,7 +27779,7 @@
       <c r="C752" s="22" t="n">
         <v>4211</v>
       </c>
-      <c r="D752" s="32" t="s">
+      <c r="D752" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E752" s="22" t="n">
@@ -27819,7 +27808,7 @@
       <c r="C753" s="24" t="s">
         <v>1340</v>
       </c>
-      <c r="D753" s="32"/>
+      <c r="D753" s="31"/>
       <c r="E753" s="22"/>
       <c r="G753" s="22" t="s">
         <v>117</v>
@@ -27835,7 +27824,7 @@
       <c r="C754" s="22" t="n">
         <v>4220</v>
       </c>
-      <c r="D754" s="32" t="s">
+      <c r="D754" s="31" t="s">
         <v>440</v>
       </c>
       <c r="E754" s="22"/>
@@ -27856,7 +27845,7 @@
       <c r="C755" s="22" t="n">
         <v>4300</v>
       </c>
-      <c r="D755" s="32" t="s">
+      <c r="D755" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E755" s="22" t="n">
@@ -27885,7 +27874,7 @@
       <c r="C756" s="22" t="n">
         <v>4301</v>
       </c>
-      <c r="D756" s="32" t="s">
+      <c r="D756" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E756" s="22" t="n">
@@ -27914,7 +27903,7 @@
       <c r="C757" s="22" t="n">
         <v>4302</v>
       </c>
-      <c r="D757" s="32" t="s">
+      <c r="D757" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E757" s="22" t="n">
@@ -27943,7 +27932,7 @@
       <c r="C758" s="22" t="n">
         <v>4303</v>
       </c>
-      <c r="D758" s="32" t="s">
+      <c r="D758" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E758" s="22" t="n">
@@ -27972,7 +27961,7 @@
       <c r="C759" s="22" t="n">
         <v>4304</v>
       </c>
-      <c r="D759" s="32" t="s">
+      <c r="D759" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E759" s="22" t="n">
@@ -28001,7 +27990,7 @@
       <c r="C760" s="22" t="n">
         <v>4306</v>
       </c>
-      <c r="D760" s="32" t="s">
+      <c r="D760" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E760" s="22" t="n">
@@ -28030,7 +28019,7 @@
       <c r="C761" s="22" t="n">
         <v>4307</v>
       </c>
-      <c r="D761" s="32" t="s">
+      <c r="D761" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E761" s="22" t="n">
@@ -28059,7 +28048,7 @@
       <c r="C762" s="22" t="n">
         <v>4308</v>
       </c>
-      <c r="D762" s="32" t="s">
+      <c r="D762" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E762" s="22" t="n">
@@ -28088,7 +28077,7 @@
       <c r="C763" s="22" t="n">
         <v>4309</v>
       </c>
-      <c r="D763" s="32" t="s">
+      <c r="D763" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E763" s="22" t="n">
@@ -28117,7 +28106,7 @@
       <c r="C764" s="22" t="n">
         <v>4310</v>
       </c>
-      <c r="D764" s="32" t="s">
+      <c r="D764" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E764" s="22" t="n">
@@ -28146,7 +28135,7 @@
       <c r="C765" s="22" t="n">
         <v>4311</v>
       </c>
-      <c r="D765" s="32" t="s">
+      <c r="D765" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E765" s="22" t="n">
@@ -28175,7 +28164,7 @@
       <c r="C766" s="24" t="s">
         <v>1344</v>
       </c>
-      <c r="D766" s="32"/>
+      <c r="D766" s="31"/>
       <c r="E766" s="22"/>
       <c r="G766" s="22" t="s">
         <v>117</v>
@@ -28191,7 +28180,7 @@
       <c r="C767" s="22" t="n">
         <v>4320</v>
       </c>
-      <c r="D767" s="32" t="s">
+      <c r="D767" s="31" t="s">
         <v>440</v>
       </c>
       <c r="E767" s="22"/>
@@ -28212,7 +28201,7 @@
       <c r="C768" s="22" t="n">
         <v>4400</v>
       </c>
-      <c r="D768" s="32" t="s">
+      <c r="D768" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E768" s="22" t="n">
@@ -28241,7 +28230,7 @@
       <c r="C769" s="22" t="n">
         <v>4401</v>
       </c>
-      <c r="D769" s="32" t="s">
+      <c r="D769" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E769" s="22" t="n">
@@ -28270,7 +28259,7 @@
       <c r="C770" s="22" t="n">
         <v>4402</v>
       </c>
-      <c r="D770" s="32" t="s">
+      <c r="D770" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E770" s="22" t="n">
@@ -28299,7 +28288,7 @@
       <c r="C771" s="22" t="n">
         <v>4403</v>
       </c>
-      <c r="D771" s="32" t="s">
+      <c r="D771" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E771" s="22" t="n">
@@ -28328,7 +28317,7 @@
       <c r="C772" s="22" t="n">
         <v>4404</v>
       </c>
-      <c r="D772" s="32" t="s">
+      <c r="D772" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E772" s="22" t="n">
@@ -28357,7 +28346,7 @@
       <c r="C773" s="22" t="n">
         <v>4406</v>
       </c>
-      <c r="D773" s="32" t="s">
+      <c r="D773" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E773" s="22" t="n">
@@ -28386,7 +28375,7 @@
       <c r="C774" s="22" t="n">
         <v>4408</v>
       </c>
-      <c r="D774" s="32" t="s">
+      <c r="D774" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E774" s="22" t="n">
@@ -28415,7 +28404,7 @@
       <c r="C775" s="22" t="n">
         <v>4409</v>
       </c>
-      <c r="D775" s="32" t="s">
+      <c r="D775" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E775" s="22" t="n">
@@ -28444,7 +28433,7 @@
       <c r="C776" s="22" t="n">
         <v>4410</v>
       </c>
-      <c r="D776" s="32" t="s">
+      <c r="D776" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E776" s="22" t="n">
@@ -28473,7 +28462,7 @@
       <c r="C777" s="22" t="n">
         <v>4411</v>
       </c>
-      <c r="D777" s="32" t="s">
+      <c r="D777" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E777" s="22" t="n">
@@ -28502,7 +28491,7 @@
       <c r="C778" s="22" t="n">
         <v>4412</v>
       </c>
-      <c r="D778" s="32" t="s">
+      <c r="D778" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E778" s="22" t="n">
@@ -28531,7 +28520,7 @@
       <c r="C779" s="22" t="n">
         <v>4413</v>
       </c>
-      <c r="D779" s="32" t="s">
+      <c r="D779" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E779" s="22" t="n">
@@ -28560,7 +28549,7 @@
       <c r="C780" s="24" t="s">
         <v>1347</v>
       </c>
-      <c r="D780" s="32"/>
+      <c r="D780" s="31"/>
       <c r="E780" s="22"/>
       <c r="G780" s="22" t="s">
         <v>117</v>
@@ -28576,7 +28565,7 @@
       <c r="C781" s="22" t="n">
         <v>4420</v>
       </c>
-      <c r="D781" s="32" t="s">
+      <c r="D781" s="31" t="s">
         <v>440</v>
       </c>
       <c r="E781" s="22"/>
@@ -28597,7 +28586,7 @@
       <c r="C782" s="22" t="n">
         <v>4500</v>
       </c>
-      <c r="D782" s="32" t="s">
+      <c r="D782" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E782" s="22" t="n">
@@ -28626,7 +28615,7 @@
       <c r="C783" s="22" t="n">
         <v>4501</v>
       </c>
-      <c r="D783" s="32" t="s">
+      <c r="D783" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E783" s="22" t="n">
@@ -28655,7 +28644,7 @@
       <c r="C784" s="22" t="n">
         <v>4502</v>
       </c>
-      <c r="D784" s="32" t="s">
+      <c r="D784" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E784" s="22" t="n">
@@ -28684,7 +28673,7 @@
       <c r="C785" s="22" t="n">
         <v>4503</v>
       </c>
-      <c r="D785" s="32" t="s">
+      <c r="D785" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E785" s="22" t="n">
@@ -28713,7 +28702,7 @@
       <c r="C786" s="22" t="n">
         <v>4504</v>
       </c>
-      <c r="D786" s="32" t="s">
+      <c r="D786" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E786" s="22" t="n">
@@ -28742,7 +28731,7 @@
       <c r="C787" s="22" t="n">
         <v>4505</v>
       </c>
-      <c r="D787" s="32" t="s">
+      <c r="D787" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E787" s="22" t="n">
@@ -28771,7 +28760,7 @@
       <c r="C788" s="22" t="n">
         <v>4506</v>
       </c>
-      <c r="D788" s="32" t="s">
+      <c r="D788" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E788" s="22" t="s">
@@ -28800,7 +28789,7 @@
       <c r="C789" s="22" t="n">
         <v>4507</v>
       </c>
-      <c r="D789" s="32" t="s">
+      <c r="D789" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E789" s="22" t="s">
@@ -28829,7 +28818,7 @@
       <c r="C790" s="22" t="n">
         <v>4508</v>
       </c>
-      <c r="D790" s="32" t="s">
+      <c r="D790" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E790" s="22" t="s">
@@ -28858,7 +28847,7 @@
       <c r="C791" s="22" t="n">
         <v>4509</v>
       </c>
-      <c r="D791" s="32" t="s">
+      <c r="D791" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E791" s="22" t="n">
@@ -28884,7 +28873,7 @@
       <c r="C792" s="22" t="n">
         <v>4510</v>
       </c>
-      <c r="D792" s="32" t="s">
+      <c r="D792" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E792" s="22" t="n">
@@ -28913,7 +28902,7 @@
       <c r="C793" s="22" t="n">
         <v>4511</v>
       </c>
-      <c r="D793" s="32" t="s">
+      <c r="D793" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E793" s="22" t="n">
@@ -28942,7 +28931,7 @@
       <c r="C794" s="22" t="n">
         <v>4512</v>
       </c>
-      <c r="D794" s="32" t="s">
+      <c r="D794" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E794" s="22" t="n">
@@ -28971,7 +28960,7 @@
       <c r="C795" s="22" t="n">
         <v>4513</v>
       </c>
-      <c r="D795" s="32" t="s">
+      <c r="D795" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E795" s="22" t="n">
@@ -29000,7 +28989,7 @@
       <c r="C796" s="22" t="n">
         <v>4514</v>
       </c>
-      <c r="D796" s="32" t="s">
+      <c r="D796" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E796" s="22" t="n">
@@ -29029,7 +29018,7 @@
       <c r="C797" s="22" t="n">
         <v>4515</v>
       </c>
-      <c r="D797" s="32" t="s">
+      <c r="D797" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E797" s="22" t="n">
@@ -29058,7 +29047,7 @@
       <c r="C798" s="22" t="n">
         <v>4516</v>
       </c>
-      <c r="D798" s="32" t="s">
+      <c r="D798" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E798" s="22" t="s">
@@ -29087,7 +29076,7 @@
       <c r="C799" s="22" t="n">
         <v>4517</v>
       </c>
-      <c r="D799" s="32" t="s">
+      <c r="D799" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E799" s="22" t="s">
@@ -29116,7 +29105,7 @@
       <c r="C800" s="22" t="n">
         <v>4518</v>
       </c>
-      <c r="D800" s="32" t="s">
+      <c r="D800" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E800" s="22" t="s">
@@ -29145,7 +29134,7 @@
       <c r="C801" s="22" t="n">
         <v>4519</v>
       </c>
-      <c r="D801" s="32" t="s">
+      <c r="D801" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E801" s="22" t="n">
@@ -29174,7 +29163,7 @@
       <c r="C802" s="22" t="n">
         <v>4520</v>
       </c>
-      <c r="D802" s="32" t="s">
+      <c r="D802" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E802" s="22" t="n">
@@ -29203,7 +29192,7 @@
       <c r="C803" s="22" t="n">
         <v>4521</v>
       </c>
-      <c r="D803" s="32" t="s">
+      <c r="D803" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E803" s="22" t="n">
@@ -29232,7 +29221,7 @@
       <c r="C804" s="22" t="n">
         <v>4522</v>
       </c>
-      <c r="D804" s="32" t="s">
+      <c r="D804" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E804" s="22" t="n">
@@ -29261,7 +29250,7 @@
       <c r="C805" s="22" t="n">
         <v>4523</v>
       </c>
-      <c r="D805" s="32" t="s">
+      <c r="D805" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E805" s="22" t="n">
@@ -29290,7 +29279,7 @@
       <c r="C806" s="22" t="n">
         <v>4524</v>
       </c>
-      <c r="D806" s="32" t="s">
+      <c r="D806" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E806" s="22" t="n">
@@ -29319,7 +29308,7 @@
       <c r="C807" s="22" t="n">
         <v>4525</v>
       </c>
-      <c r="D807" s="32" t="s">
+      <c r="D807" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E807" s="22" t="n">
@@ -29348,7 +29337,7 @@
       <c r="C808" s="22" t="n">
         <v>4526</v>
       </c>
-      <c r="D808" s="32" t="s">
+      <c r="D808" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E808" s="22" t="n">
@@ -29377,7 +29366,7 @@
       <c r="C809" s="22" t="n">
         <v>4527</v>
       </c>
-      <c r="D809" s="32" t="s">
+      <c r="D809" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E809" s="22" t="n">
@@ -29406,7 +29395,7 @@
       <c r="C810" s="22" t="n">
         <v>4528</v>
       </c>
-      <c r="D810" s="32" t="s">
+      <c r="D810" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E810" s="22" t="n">
@@ -29435,7 +29424,7 @@
       <c r="C811" s="22" t="n">
         <v>4529</v>
       </c>
-      <c r="D811" s="32" t="s">
+      <c r="D811" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E811" s="22" t="n">
@@ -29464,7 +29453,7 @@
       <c r="C812" s="22" t="n">
         <v>4530</v>
       </c>
-      <c r="D812" s="32" t="s">
+      <c r="D812" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E812" s="22" t="n">
@@ -29493,7 +29482,7 @@
       <c r="C813" s="22" t="n">
         <v>4531</v>
       </c>
-      <c r="D813" s="32" t="s">
+      <c r="D813" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E813" s="22" t="n">
@@ -29522,7 +29511,7 @@
       <c r="C814" s="22" t="n">
         <v>4532</v>
       </c>
-      <c r="D814" s="32" t="s">
+      <c r="D814" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E814" s="22" t="n">
@@ -29551,7 +29540,7 @@
       <c r="C815" s="22" t="n">
         <v>4533</v>
       </c>
-      <c r="D815" s="32" t="s">
+      <c r="D815" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E815" s="22" t="n">
@@ -29580,7 +29569,7 @@
       <c r="C816" s="22" t="n">
         <v>4534</v>
       </c>
-      <c r="D816" s="32" t="s">
+      <c r="D816" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E816" s="22" t="n">
@@ -29609,7 +29598,7 @@
       <c r="C817" s="22" t="n">
         <v>4535</v>
       </c>
-      <c r="D817" s="32" t="s">
+      <c r="D817" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E817" s="22" t="n">
@@ -29638,7 +29627,7 @@
       <c r="C818" s="22" t="n">
         <v>4536</v>
       </c>
-      <c r="D818" s="32" t="s">
+      <c r="D818" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E818" s="22" t="n">
@@ -29667,7 +29656,7 @@
       <c r="C819" s="22" t="n">
         <v>4537</v>
       </c>
-      <c r="D819" s="32" t="s">
+      <c r="D819" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E819" s="22" t="n">
@@ -29696,7 +29685,7 @@
       <c r="C820" s="22" t="n">
         <v>4538</v>
       </c>
-      <c r="D820" s="32" t="s">
+      <c r="D820" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E820" s="22" t="n">
@@ -29725,7 +29714,7 @@
       <c r="C821" s="22" t="n">
         <v>4539</v>
       </c>
-      <c r="D821" s="32" t="s">
+      <c r="D821" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E821" s="22" t="n">
@@ -29754,7 +29743,7 @@
       <c r="C822" s="22" t="n">
         <v>4540</v>
       </c>
-      <c r="D822" s="32" t="s">
+      <c r="D822" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E822" s="22" t="n">
@@ -29783,7 +29772,7 @@
       <c r="C823" s="22" t="n">
         <v>4541</v>
       </c>
-      <c r="D823" s="32" t="s">
+      <c r="D823" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E823" s="22" t="n">
@@ -29812,7 +29801,7 @@
       <c r="C824" s="22" t="n">
         <v>4542</v>
       </c>
-      <c r="D824" s="32" t="s">
+      <c r="D824" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E824" s="22" t="n">
@@ -29841,7 +29830,7 @@
       <c r="C825" s="22" t="n">
         <v>4543</v>
       </c>
-      <c r="D825" s="32" t="s">
+      <c r="D825" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E825" s="22" t="n">
@@ -29870,7 +29859,7 @@
       <c r="C826" s="22" t="n">
         <v>4544</v>
       </c>
-      <c r="D826" s="32" t="s">
+      <c r="D826" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E826" s="22" t="n">
@@ -29899,7 +29888,7 @@
       <c r="C827" s="22" t="n">
         <v>4545</v>
       </c>
-      <c r="D827" s="32" t="s">
+      <c r="D827" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E827" s="22" t="n">
@@ -29928,7 +29917,7 @@
       <c r="C828" s="22" t="n">
         <v>4546</v>
       </c>
-      <c r="D828" s="32" t="s">
+      <c r="D828" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E828" s="22" t="n">
@@ -29957,7 +29946,7 @@
       <c r="C829" s="22" t="n">
         <v>4548</v>
       </c>
-      <c r="D829" s="32" t="s">
+      <c r="D829" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E829" s="22" t="n">
@@ -29986,7 +29975,7 @@
       <c r="C830" s="22" t="n">
         <v>4550</v>
       </c>
-      <c r="D830" s="32" t="s">
+      <c r="D830" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E830" s="22" t="n">
@@ -30015,7 +30004,7 @@
       <c r="C831" s="22" t="n">
         <v>4552</v>
       </c>
-      <c r="D831" s="32" t="s">
+      <c r="D831" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E831" s="22" t="n">
@@ -30044,7 +30033,7 @@
       <c r="C832" s="22" t="n">
         <v>4554</v>
       </c>
-      <c r="D832" s="32" t="s">
+      <c r="D832" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E832" s="22" t="n">
@@ -30073,7 +30062,7 @@
       <c r="C833" s="22" t="n">
         <v>4556</v>
       </c>
-      <c r="D833" s="32" t="s">
+      <c r="D833" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E833" s="22" t="n">
@@ -30102,7 +30091,7 @@
       <c r="C834" s="22" t="n">
         <v>4558</v>
       </c>
-      <c r="D834" s="32" t="s">
+      <c r="D834" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E834" s="22" t="n">
@@ -30131,7 +30120,7 @@
       <c r="C835" s="22" t="n">
         <v>4560</v>
       </c>
-      <c r="D835" s="32" t="s">
+      <c r="D835" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E835" s="22" t="n">
@@ -30160,7 +30149,7 @@
       <c r="C836" s="22" t="n">
         <v>4562</v>
       </c>
-      <c r="D836" s="32" t="s">
+      <c r="D836" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E836" s="22" t="n">
@@ -30189,7 +30178,7 @@
       <c r="C837" s="22" t="n">
         <v>4564</v>
       </c>
-      <c r="D837" s="32" t="s">
+      <c r="D837" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E837" s="22" t="n">
@@ -30218,7 +30207,7 @@
       <c r="C838" s="22" t="n">
         <v>4566</v>
       </c>
-      <c r="D838" s="32" t="s">
+      <c r="D838" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E838" s="22" t="n">
@@ -30247,7 +30236,7 @@
       <c r="C839" s="22" t="n">
         <v>4568</v>
       </c>
-      <c r="D839" s="32" t="s">
+      <c r="D839" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E839" s="22" t="n">
@@ -30276,7 +30265,7 @@
       <c r="C840" s="22" t="n">
         <v>4570</v>
       </c>
-      <c r="D840" s="32" t="s">
+      <c r="D840" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E840" s="22" t="n">
@@ -30305,7 +30294,7 @@
       <c r="C841" s="22" t="n">
         <v>4572</v>
       </c>
-      <c r="D841" s="32" t="s">
+      <c r="D841" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E841" s="22" t="n">
@@ -30334,7 +30323,7 @@
       <c r="C842" s="22" t="n">
         <v>4574</v>
       </c>
-      <c r="D842" s="32" t="s">
+      <c r="D842" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E842" s="22" t="n">
@@ -30363,7 +30352,7 @@
       <c r="C843" s="22" t="n">
         <v>4575</v>
       </c>
-      <c r="D843" s="32" t="s">
+      <c r="D843" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E843" s="22" t="n">
@@ -30392,7 +30381,7 @@
       <c r="C844" s="22" t="n">
         <v>4576</v>
       </c>
-      <c r="D844" s="32" t="s">
+      <c r="D844" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E844" s="22" t="n">
@@ -30421,7 +30410,7 @@
       <c r="C845" s="22" t="n">
         <v>4577</v>
       </c>
-      <c r="D845" s="32" t="s">
+      <c r="D845" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E845" s="1" t="n">
@@ -30450,7 +30439,7 @@
       <c r="C846" s="22" t="n">
         <v>4578</v>
       </c>
-      <c r="D846" s="32" t="s">
+      <c r="D846" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E846" s="22" t="n">
@@ -30483,7 +30472,7 @@
       <c r="C847" s="22" t="n">
         <v>4579</v>
       </c>
-      <c r="D847" s="32" t="s">
+      <c r="D847" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E847" s="22" t="n">
@@ -30516,7 +30505,7 @@
       <c r="C848" s="22" t="n">
         <v>4580</v>
       </c>
-      <c r="D848" s="32" t="s">
+      <c r="D848" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E848" s="22" t="n">
@@ -30549,7 +30538,7 @@
       <c r="C849" s="22" t="n">
         <v>4581</v>
       </c>
-      <c r="D849" s="32" t="s">
+      <c r="D849" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E849" s="22" t="n">
@@ -30582,7 +30571,7 @@
       <c r="C850" s="22" t="n">
         <v>4582</v>
       </c>
-      <c r="D850" s="32" t="s">
+      <c r="D850" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E850" s="22" t="n">
@@ -30615,7 +30604,7 @@
       <c r="C851" s="22" t="n">
         <v>4583</v>
       </c>
-      <c r="D851" s="32" t="s">
+      <c r="D851" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E851" s="22" t="n">
@@ -30648,7 +30637,7 @@
       <c r="C852" s="22" t="n">
         <v>4584</v>
       </c>
-      <c r="D852" s="32" t="s">
+      <c r="D852" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E852" s="22" t="n">
@@ -30681,7 +30670,7 @@
       <c r="C853" s="22" t="n">
         <v>4585</v>
       </c>
-      <c r="D853" s="32" t="s">
+      <c r="D853" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E853" s="22" t="n">
@@ -30714,7 +30703,7 @@
       <c r="C854" s="22" t="n">
         <v>4586</v>
       </c>
-      <c r="D854" s="32" t="s">
+      <c r="D854" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E854" s="22" t="n">
@@ -30747,7 +30736,7 @@
       <c r="C855" s="22" t="n">
         <v>4587</v>
       </c>
-      <c r="D855" s="32" t="s">
+      <c r="D855" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E855" s="22" t="n">
@@ -30780,7 +30769,7 @@
       <c r="C856" s="22" t="n">
         <v>4588</v>
       </c>
-      <c r="D856" s="32" t="s">
+      <c r="D856" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E856" s="22" t="n">
@@ -30813,7 +30802,7 @@
       <c r="C857" s="22" t="n">
         <v>4589</v>
       </c>
-      <c r="D857" s="32" t="s">
+      <c r="D857" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E857" s="22" t="n">
@@ -30846,7 +30835,7 @@
       <c r="C858" s="22" t="n">
         <v>4590</v>
       </c>
-      <c r="D858" s="32" t="s">
+      <c r="D858" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E858" s="22" t="n">
@@ -30879,7 +30868,7 @@
       <c r="C859" s="22" t="n">
         <v>4591</v>
       </c>
-      <c r="D859" s="32" t="s">
+      <c r="D859" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E859" s="22" t="n">
@@ -30912,7 +30901,7 @@
       <c r="C860" s="22" t="n">
         <v>4592</v>
       </c>
-      <c r="D860" s="32" t="s">
+      <c r="D860" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E860" s="22" t="n">
@@ -30945,7 +30934,7 @@
       <c r="C861" s="22" t="n">
         <v>4593</v>
       </c>
-      <c r="D861" s="32" t="s">
+      <c r="D861" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E861" s="22" t="n">
@@ -30978,7 +30967,7 @@
       <c r="C862" s="1" t="n">
         <v>4594</v>
       </c>
-      <c r="D862" s="32" t="s">
+      <c r="D862" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E862" s="1" t="n">
@@ -31007,7 +30996,7 @@
       <c r="C863" s="1" t="n">
         <v>4595</v>
       </c>
-      <c r="D863" s="32" t="s">
+      <c r="D863" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E863" s="1" t="n">
@@ -31036,7 +31025,7 @@
       <c r="C864" s="1" t="n">
         <v>4596</v>
       </c>
-      <c r="D864" s="32" t="s">
+      <c r="D864" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E864" s="1" t="n">
@@ -31065,7 +31054,7 @@
       <c r="C865" s="1" t="n">
         <v>4597</v>
       </c>
-      <c r="D865" s="32" t="s">
+      <c r="D865" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E865" s="1" t="n">
@@ -31094,7 +31083,7 @@
       <c r="C866" s="1" t="n">
         <v>4598</v>
       </c>
-      <c r="D866" s="32" t="s">
+      <c r="D866" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E866" s="1" t="n">
@@ -31123,7 +31112,7 @@
       <c r="C867" s="1" t="n">
         <v>4599</v>
       </c>
-      <c r="D867" s="32" t="s">
+      <c r="D867" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E867" s="1" t="n">
@@ -31152,7 +31141,7 @@
       <c r="C868" s="1" t="n">
         <v>4600</v>
       </c>
-      <c r="D868" s="32" t="s">
+      <c r="D868" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E868" s="1" t="n">
@@ -31181,7 +31170,7 @@
       <c r="C869" s="1" t="n">
         <v>4601</v>
       </c>
-      <c r="D869" s="32" t="s">
+      <c r="D869" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E869" s="1" t="n">
@@ -31210,7 +31199,7 @@
       <c r="C870" s="1" t="n">
         <v>4602</v>
       </c>
-      <c r="D870" s="32" t="s">
+      <c r="D870" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E870" s="1" t="n">
@@ -31271,7 +31260,7 @@
       <c r="C872" s="1" t="n">
         <v>4605</v>
       </c>
-      <c r="D872" s="32" t="s">
+      <c r="D872" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E872" s="1" t="n">
@@ -31300,7 +31289,7 @@
       <c r="C873" s="1" t="n">
         <v>4606</v>
       </c>
-      <c r="D873" s="32" t="s">
+      <c r="D873" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E873" s="1" t="n">
@@ -31329,7 +31318,7 @@
       <c r="C874" s="1" t="n">
         <v>4607</v>
       </c>
-      <c r="D874" s="32" t="s">
+      <c r="D874" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E874" s="1" t="n">
@@ -31358,7 +31347,7 @@
       <c r="C875" s="1" t="n">
         <v>4608</v>
       </c>
-      <c r="D875" s="32" t="s">
+      <c r="D875" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E875" s="1" t="n">
@@ -31387,7 +31376,7 @@
       <c r="C876" s="1" t="n">
         <v>4609</v>
       </c>
-      <c r="D876" s="32" t="s">
+      <c r="D876" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E876" s="1" t="n">
@@ -31416,7 +31405,7 @@
       <c r="C877" s="1" t="n">
         <v>4610</v>
       </c>
-      <c r="D877" s="32" t="s">
+      <c r="D877" s="31" t="s">
         <v>136</v>
       </c>
       <c r="E877" s="1" t="n">
@@ -31445,7 +31434,7 @@
       <c r="C878" s="1" t="n">
         <v>4612</v>
       </c>
-      <c r="D878" s="32" t="s">
+      <c r="D878" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E878" s="1" t="n">
@@ -31474,7 +31463,7 @@
       <c r="C879" s="1" t="n">
         <v>4613</v>
       </c>
-      <c r="D879" s="32" t="s">
+      <c r="D879" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E879" s="1" t="n">
@@ -31503,7 +31492,7 @@
       <c r="C880" s="1" t="n">
         <v>4614</v>
       </c>
-      <c r="D880" s="32" t="s">
+      <c r="D880" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E880" s="1" t="n">
@@ -31532,7 +31521,7 @@
       <c r="C881" s="1" t="n">
         <v>4615</v>
       </c>
-      <c r="D881" s="32" t="s">
+      <c r="D881" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E881" s="1" t="n">
@@ -31561,7 +31550,7 @@
       <c r="C882" s="23" t="s">
         <v>1409</v>
       </c>
-      <c r="D882" s="32"/>
+      <c r="D882" s="31"/>
     </row>
     <row r="883" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A883" s="1" t="s">
@@ -31573,7 +31562,7 @@
       <c r="C883" s="1" t="n">
         <v>4620</v>
       </c>
-      <c r="D883" s="32" t="s">
+      <c r="D883" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E883" s="22" t="n">
@@ -31602,7 +31591,7 @@
       <c r="C884" s="1" t="n">
         <v>4621</v>
       </c>
-      <c r="D884" s="32"/>
+      <c r="D884" s="31"/>
       <c r="E884" s="22"/>
       <c r="G884" s="22" t="s">
         <v>117</v>
@@ -31620,7 +31609,7 @@
       <c r="C885" s="1" t="n">
         <v>4622</v>
       </c>
-      <c r="D885" s="32" t="s">
+      <c r="D885" s="31" t="s">
         <v>440</v>
       </c>
       <c r="E885" s="22"/>
@@ -31758,7 +31747,7 @@
       <c r="C890" s="1" t="n">
         <v>4700</v>
       </c>
-      <c r="D890" s="32" t="s">
+      <c r="D890" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E890" s="1" t="n">
@@ -31787,7 +31776,7 @@
       <c r="C891" s="1" t="n">
         <v>4701</v>
       </c>
-      <c r="D891" s="32" t="s">
+      <c r="D891" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E891" s="1" t="n">
@@ -31816,7 +31805,7 @@
       <c r="C892" s="1" t="n">
         <v>4702</v>
       </c>
-      <c r="D892" s="32" t="s">
+      <c r="D892" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E892" s="1" t="n">
@@ -31845,7 +31834,7 @@
       <c r="C893" s="1" t="n">
         <v>4703</v>
       </c>
-      <c r="D893" s="32" t="s">
+      <c r="D893" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E893" s="1" t="n">
@@ -31874,7 +31863,7 @@
       <c r="C894" s="1" t="n">
         <v>4704</v>
       </c>
-      <c r="D894" s="32" t="s">
+      <c r="D894" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E894" s="1" t="n">
@@ -31903,7 +31892,7 @@
       <c r="C895" s="22" t="n">
         <v>4800</v>
       </c>
-      <c r="D895" s="32" t="s">
+      <c r="D895" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E895" s="22" t="n">
@@ -31929,7 +31918,7 @@
       <c r="C896" s="22" t="n">
         <v>4801</v>
       </c>
-      <c r="D896" s="32" t="s">
+      <c r="D896" s="31" t="s">
         <v>155</v>
       </c>
       <c r="E896" s="22" t="n">
@@ -31955,7 +31944,7 @@
       <c r="C897" s="22" t="n">
         <v>4803</v>
       </c>
-      <c r="D897" s="32" t="s">
+      <c r="D897" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E897" s="22" t="n">
@@ -31984,7 +31973,7 @@
       <c r="C898" s="22" t="n">
         <v>4804</v>
       </c>
-      <c r="D898" s="32" t="s">
+      <c r="D898" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E898" s="22" t="n">
@@ -32013,7 +32002,7 @@
       <c r="C899" s="22" t="n">
         <v>4805</v>
       </c>
-      <c r="D899" s="32" t="s">
+      <c r="D899" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E899" s="22" t="n">
@@ -32042,7 +32031,7 @@
       <c r="C900" s="22" t="n">
         <v>4806</v>
       </c>
-      <c r="D900" s="32" t="s">
+      <c r="D900" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E900" s="22" t="n">
@@ -32071,7 +32060,7 @@
       <c r="C901" s="22" t="n">
         <v>4807</v>
       </c>
-      <c r="D901" s="32" t="s">
+      <c r="D901" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E901" s="22" t="n">
@@ -32100,7 +32089,7 @@
       <c r="C902" s="22" t="n">
         <v>4808</v>
       </c>
-      <c r="D902" s="32" t="s">
+      <c r="D902" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E902" s="22" t="n">
@@ -32129,7 +32118,7 @@
       <c r="C903" s="22" t="n">
         <v>4809</v>
       </c>
-      <c r="D903" s="32" t="s">
+      <c r="D903" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E903" s="22" t="n">
@@ -32158,7 +32147,7 @@
       <c r="C904" s="22" t="n">
         <v>4810</v>
       </c>
-      <c r="D904" s="32" t="s">
+      <c r="D904" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E904" s="22" t="n">
@@ -32187,7 +32176,7 @@
       <c r="C905" s="22" t="n">
         <v>4811</v>
       </c>
-      <c r="D905" s="32" t="s">
+      <c r="D905" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E905" s="22" t="n">
@@ -32216,7 +32205,7 @@
       <c r="C906" s="24" t="s">
         <v>1426</v>
       </c>
-      <c r="D906" s="32"/>
+      <c r="D906" s="31"/>
       <c r="E906" s="22"/>
       <c r="G906" s="22" t="s">
         <v>117</v>
@@ -32233,7 +32222,7 @@
       <c r="C907" s="22" t="n">
         <v>4820</v>
       </c>
-      <c r="D907" s="32" t="s">
+      <c r="D907" s="31" t="s">
         <v>440</v>
       </c>
       <c r="E907" s="22"/>
@@ -32255,7 +32244,7 @@
       <c r="C908" s="22" t="n">
         <v>4900</v>
       </c>
-      <c r="D908" s="32" t="s">
+      <c r="D908" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E908" s="22" t="n">
@@ -32284,7 +32273,7 @@
       <c r="C909" s="22" t="n">
         <v>4901</v>
       </c>
-      <c r="D909" s="32" t="s">
+      <c r="D909" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E909" s="22" t="n">
@@ -32313,7 +32302,7 @@
       <c r="C910" s="22" t="n">
         <v>4902</v>
       </c>
-      <c r="D910" s="32" t="s">
+      <c r="D910" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E910" s="22" t="n">
@@ -32342,7 +32331,7 @@
       <c r="C911" s="22" t="n">
         <v>4903</v>
       </c>
-      <c r="D911" s="32" t="s">
+      <c r="D911" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E911" s="22" t="n">
@@ -32371,7 +32360,7 @@
       <c r="C912" s="22" t="n">
         <v>4904</v>
       </c>
-      <c r="D912" s="32" t="s">
+      <c r="D912" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E912" s="22" t="n">
@@ -32400,7 +32389,7 @@
       <c r="C913" s="22" t="n">
         <v>4905</v>
       </c>
-      <c r="D913" s="32" t="s">
+      <c r="D913" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E913" s="22" t="n">
@@ -32429,7 +32418,7 @@
       <c r="C914" s="22" t="n">
         <v>4906</v>
       </c>
-      <c r="D914" s="32" t="s">
+      <c r="D914" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E914" s="22" t="n">
@@ -32458,7 +32447,7 @@
       <c r="C915" s="22" t="n">
         <v>4907</v>
       </c>
-      <c r="D915" s="32" t="s">
+      <c r="D915" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E915" s="22" t="s">
@@ -32487,7 +32476,7 @@
       <c r="C916" s="22" t="n">
         <v>4908</v>
       </c>
-      <c r="D916" s="32" t="s">
+      <c r="D916" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E916" s="22" t="s">
@@ -32516,7 +32505,7 @@
       <c r="C917" s="22" t="n">
         <v>4909</v>
       </c>
-      <c r="D917" s="32" t="s">
+      <c r="D917" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E917" s="22" t="s">
@@ -32545,7 +32534,7 @@
       <c r="C918" s="22" t="n">
         <v>4910</v>
       </c>
-      <c r="D918" s="32" t="s">
+      <c r="D918" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E918" s="22" t="n">
@@ -32574,7 +32563,7 @@
       <c r="C919" s="22" t="n">
         <v>4911</v>
       </c>
-      <c r="D919" s="32" t="s">
+      <c r="D919" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E919" s="22" t="n">
@@ -32603,7 +32592,7 @@
       <c r="C920" s="22" t="n">
         <v>4912</v>
       </c>
-      <c r="D920" s="32" t="s">
+      <c r="D920" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E920" s="22" t="n">
@@ -32632,7 +32621,7 @@
       <c r="C921" s="22" t="n">
         <v>4913</v>
       </c>
-      <c r="D921" s="32" t="s">
+      <c r="D921" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E921" s="22" t="n">
@@ -32661,7 +32650,7 @@
       <c r="C922" s="22" t="n">
         <v>4914</v>
       </c>
-      <c r="D922" s="32" t="s">
+      <c r="D922" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E922" s="22" t="n">
@@ -32690,7 +32679,7 @@
       <c r="C923" s="22" t="n">
         <v>4915</v>
       </c>
-      <c r="D923" s="32" t="s">
+      <c r="D923" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E923" s="22" t="n">
@@ -32719,7 +32708,7 @@
       <c r="C924" s="22" t="n">
         <v>4916</v>
       </c>
-      <c r="D924" s="32" t="s">
+      <c r="D924" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E924" s="22" t="n">
@@ -32748,7 +32737,7 @@
       <c r="C925" s="22" t="n">
         <v>4917</v>
       </c>
-      <c r="D925" s="32" t="s">
+      <c r="D925" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E925" s="22" t="s">
@@ -32777,7 +32766,7 @@
       <c r="C926" s="22" t="n">
         <v>4918</v>
       </c>
-      <c r="D926" s="32" t="s">
+      <c r="D926" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E926" s="22" t="s">
@@ -32806,7 +32795,7 @@
       <c r="C927" s="22" t="n">
         <v>4919</v>
       </c>
-      <c r="D927" s="32" t="s">
+      <c r="D927" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E927" s="22" t="s">
@@ -32835,7 +32824,7 @@
       <c r="C928" s="22" t="n">
         <v>4920</v>
       </c>
-      <c r="D928" s="32" t="s">
+      <c r="D928" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E928" s="22" t="n">
@@ -32864,7 +32853,7 @@
       <c r="C929" s="22" t="n">
         <v>4921</v>
       </c>
-      <c r="D929" s="32" t="s">
+      <c r="D929" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E929" s="22" t="n">
@@ -32893,7 +32882,7 @@
       <c r="C930" s="22" t="n">
         <v>4922</v>
       </c>
-      <c r="D930" s="32" t="s">
+      <c r="D930" s="31" t="s">
         <v>136</v>
       </c>
       <c r="E930" s="22" t="n">
@@ -32922,7 +32911,7 @@
       <c r="C931" s="22" t="n">
         <v>4924</v>
       </c>
-      <c r="D931" s="32" t="s">
+      <c r="D931" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E931" s="22" t="n">
@@ -32951,7 +32940,7 @@
       <c r="C932" s="1" t="n">
         <v>4925</v>
       </c>
-      <c r="D932" s="32" t="s">
+      <c r="D932" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E932" s="1" t="n">
@@ -33216,7 +33205,7 @@
       <c r="C943" s="25" t="n">
         <v>5200</v>
       </c>
-      <c r="D943" s="32" t="s">
+      <c r="D943" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E943" s="25" t="n">
@@ -33242,7 +33231,7 @@
       <c r="C944" s="25" t="n">
         <v>5201</v>
       </c>
-      <c r="D944" s="32" t="s">
+      <c r="D944" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E944" s="25" t="n">
@@ -33268,7 +33257,7 @@
       <c r="C945" s="25" t="n">
         <v>5202</v>
       </c>
-      <c r="D945" s="32" t="s">
+      <c r="D945" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E945" s="25" t="n">
@@ -33294,7 +33283,7 @@
       <c r="C946" s="25" t="n">
         <v>5203</v>
       </c>
-      <c r="D946" s="32" t="s">
+      <c r="D946" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E946" s="25" t="n">
@@ -33320,7 +33309,7 @@
       <c r="C947" s="25" t="n">
         <v>5204</v>
       </c>
-      <c r="D947" s="32" t="s">
+      <c r="D947" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E947" s="25" t="n">
@@ -33349,7 +33338,7 @@
       <c r="C948" s="25" t="n">
         <v>5205</v>
       </c>
-      <c r="D948" s="32" t="s">
+      <c r="D948" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E948" s="25" t="n">
@@ -33378,7 +33367,7 @@
       <c r="C949" s="25" t="n">
         <v>5206</v>
       </c>
-      <c r="D949" s="32" t="s">
+      <c r="D949" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E949" s="25" t="n">
@@ -33407,7 +33396,7 @@
       <c r="C950" s="25" t="n">
         <v>5207</v>
       </c>
-      <c r="D950" s="32" t="s">
+      <c r="D950" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E950" s="25" t="n">
@@ -33436,7 +33425,7 @@
       <c r="C951" s="25" t="n">
         <v>5208</v>
       </c>
-      <c r="D951" s="32" t="s">
+      <c r="D951" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E951" s="25" t="n">
@@ -33465,7 +33454,7 @@
       <c r="C952" s="25" t="n">
         <v>5209</v>
       </c>
-      <c r="D952" s="32" t="s">
+      <c r="D952" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E952" s="25" t="s">
@@ -33494,7 +33483,7 @@
       <c r="C953" s="25" t="n">
         <v>5210</v>
       </c>
-      <c r="D953" s="32" t="s">
+      <c r="D953" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E953" s="25" t="n">
@@ -33523,7 +33512,7 @@
       <c r="C954" s="25" t="n">
         <v>5211</v>
       </c>
-      <c r="D954" s="32" t="s">
+      <c r="D954" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E954" s="25" t="n">
@@ -33552,7 +33541,7 @@
       <c r="C955" s="25" t="n">
         <v>5212</v>
       </c>
-      <c r="D955" s="32" t="s">
+      <c r="D955" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E955" s="25" t="n">
@@ -33581,7 +33570,7 @@
       <c r="C956" s="25" t="n">
         <v>5213</v>
       </c>
-      <c r="D956" s="32" t="s">
+      <c r="D956" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E956" s="25" t="n">
@@ -33610,7 +33599,7 @@
       <c r="C957" s="25" t="n">
         <v>5214</v>
       </c>
-      <c r="D957" s="32" t="s">
+      <c r="D957" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E957" s="25" t="n">
@@ -33639,7 +33628,7 @@
       <c r="C958" s="25" t="n">
         <v>5215</v>
       </c>
-      <c r="D958" s="32" t="s">
+      <c r="D958" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E958" s="25" t="n">
@@ -33668,7 +33657,7 @@
       <c r="C959" s="25" t="n">
         <v>5216</v>
       </c>
-      <c r="D959" s="32" t="s">
+      <c r="D959" s="31" t="s">
         <v>59</v>
       </c>
       <c r="E959" s="25" t="n">
@@ -33697,7 +33686,7 @@
       <c r="C960" s="25" t="n">
         <v>5217</v>
       </c>
-      <c r="D960" s="32" t="s">
+      <c r="D960" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E960" s="25" t="n">
@@ -33720,7 +33709,7 @@
       <c r="C961" s="25" t="n">
         <v>5218</v>
       </c>
-      <c r="D961" s="32" t="s">
+      <c r="D961" s="31" t="s">
         <v>1168</v>
       </c>
       <c r="E961" s="25" t="n">
@@ -33746,7 +33735,7 @@
       <c r="C962" s="25" t="n">
         <v>5234</v>
       </c>
-      <c r="D962" s="32" t="s">
+      <c r="D962" s="31" t="s">
         <v>1168</v>
       </c>
       <c r="E962" s="25" t="n">
@@ -33769,7 +33758,7 @@
       <c r="C963" s="25" t="n">
         <v>5250</v>
       </c>
-      <c r="D963" s="32" t="s">
+      <c r="D963" s="31" t="s">
         <v>1168</v>
       </c>
       <c r="E963" s="25" t="n">
@@ -33792,7 +33781,7 @@
       <c r="C964" s="25" t="n">
         <v>5266</v>
       </c>
-      <c r="D964" s="32" t="s">
+      <c r="D964" s="31" t="s">
         <v>1168</v>
       </c>
       <c r="E964" s="25" t="n">
@@ -33815,7 +33804,7 @@
       <c r="C965" s="25" t="n">
         <v>5282</v>
       </c>
-      <c r="D965" s="32" t="s">
+      <c r="D965" s="31" t="s">
         <v>1168</v>
       </c>
       <c r="E965" s="25" t="n">
@@ -33838,7 +33827,7 @@
       <c r="C966" s="25" t="n">
         <v>5298</v>
       </c>
-      <c r="D966" s="32" t="s">
+      <c r="D966" s="31" t="s">
         <v>1168</v>
       </c>
       <c r="E966" s="25" t="n">
@@ -33861,7 +33850,7 @@
       <c r="C967" s="25" t="n">
         <v>5314</v>
       </c>
-      <c r="D967" s="32" t="s">
+      <c r="D967" s="31" t="s">
         <v>1168</v>
       </c>
       <c r="E967" s="25" t="n">
@@ -33884,7 +33873,7 @@
       <c r="C968" s="25" t="n">
         <v>5330</v>
       </c>
-      <c r="D968" s="32" t="s">
+      <c r="D968" s="31" t="s">
         <v>1168</v>
       </c>
       <c r="E968" s="25" t="n">
@@ -33907,7 +33896,7 @@
       <c r="C969" s="24" t="s">
         <v>1452</v>
       </c>
-      <c r="D969" s="32"/>
+      <c r="D969" s="31"/>
       <c r="E969" s="25"/>
       <c r="G969" s="25" t="s">
         <v>117</v>
@@ -33923,7 +33912,7 @@
       <c r="C970" s="25" t="n">
         <v>5350</v>
       </c>
-      <c r="D970" s="32" t="s">
+      <c r="D970" s="31" t="s">
         <v>440</v>
       </c>
       <c r="E970" s="25"/>
@@ -33944,7 +33933,7 @@
       <c r="C971" s="1" t="n">
         <v>5400</v>
       </c>
-      <c r="D971" s="32" t="s">
+      <c r="D971" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E971" s="1" t="n">
@@ -33973,7 +33962,7 @@
       <c r="C972" s="1" t="n">
         <v>5401</v>
       </c>
-      <c r="D972" s="32" t="s">
+      <c r="D972" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E972" s="1" t="n">
@@ -34002,7 +33991,7 @@
       <c r="C973" s="1" t="n">
         <v>5402</v>
       </c>
-      <c r="D973" s="32" t="s">
+      <c r="D973" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E973" s="1" t="n">
@@ -34031,7 +34020,7 @@
       <c r="C974" s="1" t="n">
         <v>5403</v>
       </c>
-      <c r="D974" s="32" t="s">
+      <c r="D974" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E974" s="1" t="n">
@@ -34057,7 +34046,7 @@
       <c r="C975" s="1" t="n">
         <v>5404</v>
       </c>
-      <c r="D975" s="32" t="s">
+      <c r="D975" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E975" s="1" t="n">
@@ -34086,7 +34075,7 @@
       <c r="C976" s="1" t="n">
         <v>5405</v>
       </c>
-      <c r="D976" s="32" t="s">
+      <c r="D976" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E976" s="1" t="n">
@@ -34115,7 +34104,7 @@
       <c r="C977" s="1" t="n">
         <v>5406</v>
       </c>
-      <c r="D977" s="32" t="s">
+      <c r="D977" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E977" s="1" t="n">
@@ -34144,7 +34133,7 @@
       <c r="C978" s="1" t="n">
         <v>5407</v>
       </c>
-      <c r="D978" s="32" t="s">
+      <c r="D978" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E978" s="1" t="n">
@@ -34173,7 +34162,7 @@
       <c r="C979" s="1" t="n">
         <v>5420</v>
       </c>
-      <c r="D979" s="32" t="s">
+      <c r="D979" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E979" s="1" t="n">
@@ -34202,7 +34191,7 @@
       <c r="C980" s="1" t="n">
         <v>5421</v>
       </c>
-      <c r="D980" s="32" t="s">
+      <c r="D980" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E980" s="1" t="n">
@@ -34231,7 +34220,7 @@
       <c r="C981" s="1" t="n">
         <v>5422</v>
       </c>
-      <c r="D981" s="32" t="s">
+      <c r="D981" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E981" s="1" t="n">
@@ -34260,7 +34249,7 @@
       <c r="C982" s="1" t="n">
         <v>5423</v>
       </c>
-      <c r="D982" s="32" t="s">
+      <c r="D982" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E982" s="1" t="n">
@@ -34289,7 +34278,7 @@
       <c r="C983" s="1" t="n">
         <v>5424</v>
       </c>
-      <c r="D983" s="32" t="s">
+      <c r="D983" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E983" s="1" t="n">
@@ -34318,7 +34307,7 @@
       <c r="C984" s="1" t="n">
         <v>5425</v>
       </c>
-      <c r="D984" s="32" t="s">
+      <c r="D984" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E984" s="1" t="n">
@@ -34347,7 +34336,7 @@
       <c r="C985" s="1" t="n">
         <v>5426</v>
       </c>
-      <c r="D985" s="32" t="s">
+      <c r="D985" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E985" s="1" t="n">
@@ -34376,7 +34365,7 @@
       <c r="C986" s="1" t="n">
         <v>5427</v>
       </c>
-      <c r="D986" s="32" t="s">
+      <c r="D986" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E986" s="1" t="n">
@@ -34431,7 +34420,7 @@
       <c r="C988" s="1" t="n">
         <v>5430</v>
       </c>
-      <c r="D988" s="32" t="s">
+      <c r="D988" s="31" t="s">
         <v>20</v>
       </c>
       <c r="E988" s="1" t="n">
@@ -34910,58 +34899,58 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="32" t="s">
         <v>1524</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="33" t="s">
         <v>1525</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="35"/>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
+      <c r="A3" s="34"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="33" t="s">
         <v>1526</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="35"/>
-      <c r="B5" s="35"/>
-      <c r="C5" s="35"/>
+      <c r="A5" s="34"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="35"/>
-      <c r="B6" s="35"/>
-      <c r="C6" s="35"/>
+      <c r="A6" s="34"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="34"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="34" t="s">
         <v>1527</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="34" t="s">
         <v>1528</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="34" t="s">
         <v>1529</v>
       </c>
     </row>
@@ -35129,24 +35118,24 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="34" t="n">
+      <c r="A28" s="33" t="n">
         <v>223</v>
       </c>
-      <c r="B28" s="34" t="n">
+      <c r="B28" s="33" t="n">
         <v>277</v>
       </c>
-      <c r="C28" s="34" t="s">
+      <c r="C28" s="33" t="s">
         <v>1531</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="34" t="n">
+      <c r="A29" s="33" t="n">
         <v>224</v>
       </c>
-      <c r="B29" s="34" t="n">
+      <c r="B29" s="33" t="n">
         <v>278</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="33" t="s">
         <v>1532</v>
       </c>
     </row>
@@ -35162,57 +35151,57 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="34" t="n">
+      <c r="A31" s="33" t="n">
         <v>226</v>
       </c>
-      <c r="B31" s="34" t="n">
+      <c r="B31" s="33" t="n">
         <v>279</v>
       </c>
-      <c r="C31" s="34" t="s">
+      <c r="C31" s="33" t="s">
         <v>1534</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="34" t="n">
+      <c r="A32" s="33" t="n">
         <v>227</v>
       </c>
-      <c r="B32" s="34" t="n">
+      <c r="B32" s="33" t="n">
         <v>276</v>
       </c>
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="33" t="s">
         <v>1535</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="34" t="n">
+      <c r="A33" s="33" t="n">
         <v>228</v>
       </c>
-      <c r="B33" s="34" t="n">
+      <c r="B33" s="33" t="n">
         <v>275</v>
       </c>
-      <c r="C33" s="34" t="s">
+      <c r="C33" s="33" t="s">
         <v>1536</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="34" t="n">
+      <c r="A34" s="33" t="n">
         <v>229</v>
       </c>
-      <c r="B34" s="34" t="n">
+      <c r="B34" s="33" t="n">
         <v>274</v>
       </c>
-      <c r="C34" s="34" t="s">
+      <c r="C34" s="33" t="s">
         <v>1537</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="34" t="n">
+      <c r="A35" s="33" t="n">
         <v>230</v>
       </c>
-      <c r="B35" s="34" t="n">
+      <c r="B35" s="33" t="n">
         <v>273</v>
       </c>
-      <c r="C35" s="34" t="s">
+      <c r="C35" s="33" t="s">
         <v>1538</v>
       </c>
     </row>
@@ -35316,35 +35305,35 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="34" t="n">
+      <c r="A45" s="33" t="n">
         <v>242</v>
       </c>
-      <c r="B45" s="34" t="n">
+      <c r="B45" s="33" t="n">
         <v>261</v>
       </c>
-      <c r="C45" s="34" t="s">
+      <c r="C45" s="33" t="s">
         <v>1548</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="34" t="n">
+      <c r="A46" s="33" t="n">
         <v>243</v>
       </c>
-      <c r="B46" s="34" t="n">
+      <c r="B46" s="33" t="n">
         <v>260</v>
       </c>
-      <c r="C46" s="34" t="s">
+      <c r="C46" s="33" t="s">
         <v>1549</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="34" t="n">
+      <c r="A47" s="33" t="n">
         <v>244</v>
       </c>
-      <c r="B47" s="34" t="n">
+      <c r="B47" s="33" t="n">
         <v>259</v>
       </c>
-      <c r="C47" s="34"/>
+      <c r="C47" s="33"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="22" t="n">
@@ -35353,7 +35342,7 @@
       <c r="B48" s="22" t="n">
         <v>258</v>
       </c>
-      <c r="C48" s="34" t="s">
+      <c r="C48" s="33" t="s">
         <v>1550</v>
       </c>
     </row>
@@ -35643,7 +35632,7 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C39" s="36" t="s">
+      <c r="C39" s="35" t="s">
         <v>1602</v>
       </c>
     </row>

</xml_diff>